<commit_message>
≡ƒÜÇ PO Status update via batch
</commit_message>
<xml_diff>
--- a/po-status.xlsx
+++ b/po-status.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esolon\OneDrive - Boston Semi Equipment LLC\Github Projects\PO_Status\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mvtstechnologies-my.sharepoint.com/personal/edsel_solon_bsegroup_com/Documents/Github Projects/PO_Status/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519F3434-12A6-47DF-98DF-6D77C031F382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_BEA61AB9CEBD7FEC0FBAFCEDFDF793F070D80A79" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1DB55FD-920A-4A06-8BFC-ABBEFCC9C9B3}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="PO_StatusQry" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="PO_StatusQry">PO_StatusQry!$A$2:$M$86</definedName>
+    <definedName name="PO_StatusQry">PO_StatusQry!$A$2:$M$99</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="171">
   <si>
     <t>CustName</t>
   </si>
@@ -70,10 +70,7 @@
     <t>4516351202_ASEWH</t>
   </si>
   <si>
-    <t>OverDue by 187 days</t>
-  </si>
-  <si>
-    <t>Varies (2025-08-29 → 2026-02-24)</t>
+    <t>OverDue by 255 days</t>
   </si>
   <si>
     <t>Texas Instruments SCT</t>
@@ -82,6 +79,9 @@
     <t>4516351202_SCT</t>
   </si>
   <si>
+    <t>Varies (2025-08-29 → 2026-05-13)</t>
+  </si>
+  <si>
     <t>Texas Instruments Taiwan</t>
   </si>
   <si>
@@ -94,16 +94,28 @@
     <t>4516351202_TICL-PR</t>
   </si>
   <si>
+    <t>Varies (2025-08-29 → 2026-05-11)</t>
+  </si>
+  <si>
     <t>TEXAS INSTRUMENTS  MALAYSIA</t>
   </si>
   <si>
     <t>Global PO 4516351202</t>
   </si>
   <si>
-    <t>OverDue by 121 days</t>
-  </si>
-  <si>
-    <t>Varies (2025-11-03 → 2026-02-24)</t>
+    <t>OverDue by 91 days</t>
+  </si>
+  <si>
+    <t>ASE ASSEMBLY AND TEST LIMITED</t>
+  </si>
+  <si>
+    <t>4516351202_ASESH</t>
+  </si>
+  <si>
+    <t>OverDue by 76 days</t>
+  </si>
+  <si>
+    <t>Varies (2026-02-24 → 2026-04-08)</t>
   </si>
   <si>
     <t>TI (Philippines) Inc.</t>
@@ -112,10 +124,22 @@
     <t>4516351202_TIPI</t>
   </si>
   <si>
-    <t>OverDue by 44 days</t>
-  </si>
-  <si>
-    <t>Varies (2026-01-19 → 2026-03-13)</t>
+    <t>OverDue by 60 days</t>
+  </si>
+  <si>
+    <t>Varies (2026-03-12 → 2026-05-19)</t>
+  </si>
+  <si>
+    <t>ARDENTEC CORPORATION</t>
+  </si>
+  <si>
+    <t>4516351202_ARD</t>
+  </si>
+  <si>
+    <t>OverDue by 45 days</t>
+  </si>
+  <si>
+    <t>Varies (2026-03-27 → 2026-05-19)</t>
   </si>
   <si>
     <t>Analog Devices Gen. Trias Inc. (ADGT)</t>
@@ -124,172 +148,118 @@
     <t>47270551</t>
   </si>
   <si>
-    <t>OverDue by 16 days</t>
-  </si>
-  <si>
-    <t>Hana Semiconductor (Ayutthaya) Co., Ltd (HNT)</t>
-  </si>
-  <si>
-    <t>4516351202_HNT</t>
-  </si>
-  <si>
-    <t>OverDue by 12 days</t>
-  </si>
-  <si>
-    <t>Texas Instruments AIZU</t>
-  </si>
-  <si>
-    <t>4516351202_AIZU</t>
-  </si>
-  <si>
-    <t>OverDue by 9 days</t>
-  </si>
-  <si>
-    <t>Varies (2026-02-23 → 2026-03-05)</t>
+    <t>OverDue by 14 days</t>
+  </si>
+  <si>
+    <t>Varies (2026-04-27 → 2026-05-13)</t>
+  </si>
+  <si>
+    <t>Lingsen Precision Industries Ltd.</t>
+  </si>
+  <si>
+    <t>4516446856</t>
+  </si>
+  <si>
+    <t>7 days before Due</t>
+  </si>
+  <si>
+    <t>NXP Malaysia Sdn. Bhd.</t>
+  </si>
+  <si>
+    <t>3T/PO262326</t>
+  </si>
+  <si>
+    <t>TEXAS INSTRUMENTS (INDIA) Pvt. Ltd</t>
+  </si>
+  <si>
+    <t>4516351202_TII</t>
+  </si>
+  <si>
+    <t>TBA_NXP</t>
+  </si>
+  <si>
+    <t>Texas Instruments LFAB</t>
+  </si>
+  <si>
+    <t>4516351202_LFAB</t>
+  </si>
+  <si>
+    <t>ROCHESTER ELECTRONICS</t>
+  </si>
+  <si>
+    <t>252395</t>
+  </si>
+  <si>
+    <t>Texas Instruments DMOS5</t>
+  </si>
+  <si>
+    <t>4516351202_DMOS5</t>
+  </si>
+  <si>
+    <t>Completed PO</t>
+  </si>
+  <si>
+    <t>47188646</t>
+  </si>
+  <si>
+    <t>47218149</t>
+  </si>
+  <si>
+    <t>47245848</t>
+  </si>
+  <si>
+    <t>47245933</t>
+  </si>
+  <si>
+    <t>47253728</t>
+  </si>
+  <si>
+    <t>47264622</t>
+  </si>
+  <si>
+    <t>47274630</t>
+  </si>
+  <si>
+    <t>47276474</t>
+  </si>
+  <si>
+    <t>47283634</t>
+  </si>
+  <si>
+    <t>47283654</t>
+  </si>
+  <si>
+    <t>47286185</t>
+  </si>
+  <si>
+    <t>47289023</t>
+  </si>
+  <si>
+    <t>47290167</t>
+  </si>
+  <si>
+    <t>47292239</t>
+  </si>
+  <si>
+    <t>47292914</t>
+  </si>
+  <si>
+    <t>47296581</t>
+  </si>
+  <si>
+    <t>47296806</t>
   </si>
   <si>
     <t>47301012</t>
   </si>
   <si>
-    <t>19 days before Due</t>
-  </si>
-  <si>
-    <t>STMicroelectronics, Inc.</t>
-  </si>
-  <si>
-    <t>4010017970</t>
-  </si>
-  <si>
-    <t>15 days before Due</t>
-  </si>
-  <si>
-    <t>Texas Instruments LFAB</t>
-  </si>
-  <si>
-    <t>4516351202_LFAB</t>
-  </si>
-  <si>
-    <t>12 days before Due</t>
-  </si>
-  <si>
-    <t>UTAC Thai Limited ( UTL 3)</t>
-  </si>
-  <si>
-    <t>4516351202_UTL</t>
-  </si>
-  <si>
-    <t>2 days before Due</t>
-  </si>
-  <si>
-    <t>TI Philippines, Inc - Clark FT</t>
-  </si>
-  <si>
-    <t>4516351202_TICL-FT</t>
-  </si>
-  <si>
-    <t>Due Today</t>
-  </si>
-  <si>
-    <t>ARDENTEC CORPORATION</t>
-  </si>
-  <si>
-    <t>4516351202_ARD</t>
-  </si>
-  <si>
-    <t>Texas Instruments Japan Limited MIHO Plant (MIHO 8 FAB)</t>
-  </si>
-  <si>
-    <t>4516351202_MIHO</t>
-  </si>
-  <si>
-    <t>Texas Instruments DMOS5</t>
-  </si>
-  <si>
-    <t>4516351202_DMOS5</t>
-  </si>
-  <si>
-    <t>NXP Malaysia Sdn. Bhd.</t>
-  </si>
-  <si>
-    <t>TBA_NXP</t>
-  </si>
-  <si>
-    <t>TEXAS INSTRUMENTS (INDIA) Pvt. Ltd</t>
-  </si>
-  <si>
-    <t>4516351202_TII</t>
-  </si>
-  <si>
-    <t>Texas Instruments Taiwan Limited</t>
-  </si>
-  <si>
-    <t>4516450237</t>
-  </si>
-  <si>
-    <t>ROCHESTER ELECTRONICS</t>
-  </si>
-  <si>
-    <t>252395</t>
-  </si>
-  <si>
-    <t>47188646</t>
-  </si>
-  <si>
-    <t>Completed PO</t>
-  </si>
-  <si>
-    <t>47218149</t>
-  </si>
-  <si>
-    <t>47245848</t>
-  </si>
-  <si>
-    <t>47245933</t>
-  </si>
-  <si>
-    <t>47253728</t>
-  </si>
-  <si>
-    <t>47264622</t>
-  </si>
-  <si>
-    <t>47274630</t>
-  </si>
-  <si>
-    <t>47276474</t>
-  </si>
-  <si>
-    <t>47283634</t>
-  </si>
-  <si>
-    <t>47283654</t>
-  </si>
-  <si>
-    <t>47286185</t>
-  </si>
-  <si>
-    <t>47289023</t>
-  </si>
-  <si>
-    <t>47290167</t>
-  </si>
-  <si>
-    <t>47292239</t>
-  </si>
-  <si>
-    <t>47292914</t>
-  </si>
-  <si>
-    <t>47296581</t>
-  </si>
-  <si>
-    <t>47296806</t>
-  </si>
-  <si>
     <t>47301646</t>
   </si>
   <si>
     <t>47304169</t>
+  </si>
+  <si>
+    <t>47324752</t>
   </si>
   <si>
     <t>ANALOG DEVICES INC. CAMAS</t>
@@ -311,12 +281,30 @@
     <t>8541541216</t>
   </si>
   <si>
+    <t>8541550629</t>
+  </si>
+  <si>
+    <t>8541550824</t>
+  </si>
+  <si>
+    <t>Boston Semi Equipment</t>
+  </si>
+  <si>
+    <t>TBDBSEMY</t>
+  </si>
+  <si>
     <t>Boston Semi Equipment (Thailand) Co.,Ltd.</t>
   </si>
   <si>
     <t>TBA_BSETH</t>
   </si>
   <si>
+    <t>Boston Semi Equipment Asia</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
     <t>CARDIAC PACEMAKERS INC</t>
   </si>
   <si>
@@ -332,12 +320,21 @@
     <t>7000675296</t>
   </si>
   <si>
+    <t>7000696372</t>
+  </si>
+  <si>
     <t>Hana Semiconductor (Ayutthaya) Co., Ltd</t>
   </si>
   <si>
     <t>4910173913</t>
   </si>
   <si>
+    <t>Hana Semiconductor (Ayutthaya) Co., Ltd (HNT)</t>
+  </si>
+  <si>
+    <t>4516351202_HNT</t>
+  </si>
+  <si>
     <t>4910172298</t>
   </si>
   <si>
@@ -347,15 +344,9 @@
     <t>ES072525</t>
   </si>
   <si>
-    <t>Lingsen Precision Industries Ltd.</t>
-  </si>
-  <si>
     <t>4516260169</t>
   </si>
   <si>
-    <t>4516446856</t>
-  </si>
-  <si>
     <t>LPI-2507174</t>
   </si>
   <si>
@@ -380,6 +371,21 @@
     <t>3T/PO262313</t>
   </si>
   <si>
+    <t>3T/PO262321</t>
+  </si>
+  <si>
+    <t>ON Semiconductor Philippines Inc</t>
+  </si>
+  <si>
+    <t>561000005506</t>
+  </si>
+  <si>
+    <t>Rhenus Logistics Co.,Ltd.</t>
+  </si>
+  <si>
+    <t>TBDBSETH</t>
+  </si>
+  <si>
     <t>ST Microelectronics Pte Ltd.</t>
   </si>
   <si>
@@ -389,6 +395,9 @@
     <t>4020007647</t>
   </si>
   <si>
+    <t>STMicroelectronics, Inc.</t>
+  </si>
+  <si>
     <t>3030012690</t>
   </si>
   <si>
@@ -404,6 +413,12 @@
     <t>4010017128</t>
   </si>
   <si>
+    <t>4010017970</t>
+  </si>
+  <si>
+    <t>4010018238</t>
+  </si>
+  <si>
     <t>4330007739</t>
   </si>
   <si>
@@ -419,6 +434,12 @@
     <t>BSE-58645</t>
   </si>
   <si>
+    <t>Texas Instruments AIZU</t>
+  </si>
+  <si>
+    <t>4516351202_AIZU</t>
+  </si>
+  <si>
     <t>Texas Instruments CLAB</t>
   </si>
   <si>
@@ -458,15 +479,39 @@
     <t>4516351202_MIHO-ENG</t>
   </si>
   <si>
+    <t>Texas Instruments Japan Limited MIHO Plant (MIHO 8 FAB)</t>
+  </si>
+  <si>
+    <t>4516351202_MIHO</t>
+  </si>
+  <si>
+    <t>Texas Instruments RFAB</t>
+  </si>
+  <si>
+    <t>4516351202_RFAB</t>
+  </si>
+  <si>
     <t>Texas Instruments SFAB</t>
   </si>
   <si>
     <t>4516351202_SFAB</t>
   </si>
   <si>
+    <t>Texas Instruments Taiwan Limited</t>
+  </si>
+  <si>
+    <t>4516450237</t>
+  </si>
+  <si>
     <t>4910171717</t>
   </si>
   <si>
+    <t>TI Philippines, Inc - Clark FT</t>
+  </si>
+  <si>
+    <t>4516351202_TICL-FT</t>
+  </si>
+  <si>
     <t>TKC Enterprises Inc.</t>
   </si>
   <si>
@@ -479,13 +524,19 @@
     <t>4516351202_NFME</t>
   </si>
   <si>
+    <t>UTAC Thai Limited ( UTL 3)</t>
+  </si>
+  <si>
     <t>43151446</t>
   </si>
   <si>
     <t>43156228</t>
   </si>
   <si>
-    <t>Last updated: 2026-03-04 14:06:04</t>
+    <t>4516351202_UTL</t>
+  </si>
+  <si>
+    <t>Last updated: 2026-05-11 08:55:50</t>
   </si>
 </sst>
 </file>
@@ -830,12 +881,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M99"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.5">
@@ -887,19 +938,19 @@
         <v>14</v>
       </c>
       <c r="C3">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -908,36 +959,33 @@
         <v>45898</v>
       </c>
       <c r="K3">
-        <v>-187</v>
+        <v>-255</v>
       </c>
       <c r="L3" t="s">
         <v>15</v>
       </c>
-      <c r="M3" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
       <c r="C4">
-        <v>223</v>
+        <v>270</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>220</v>
+        <v>259</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -946,10 +994,13 @@
         <v>45898</v>
       </c>
       <c r="K4">
-        <v>-187</v>
+        <v>-255</v>
       </c>
       <c r="L4" t="s">
         <v>15</v>
+      </c>
+      <c r="M4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.5">
@@ -960,19 +1011,19 @@
         <v>20</v>
       </c>
       <c r="C5">
-        <v>242</v>
+        <v>281</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>2</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H5">
-        <v>238</v>
+        <v>262</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -981,7 +1032,7 @@
         <v>45898</v>
       </c>
       <c r="K5">
-        <v>-187</v>
+        <v>-255</v>
       </c>
       <c r="L5" t="s">
         <v>15</v>
@@ -995,19 +1046,19 @@
         <v>22</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>156</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="H6">
-        <v>40</v>
+        <v>107</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1016,47 +1067,47 @@
         <v>45898</v>
       </c>
       <c r="K6">
-        <v>-187</v>
+        <v>-255</v>
       </c>
       <c r="L6" t="s">
         <v>15</v>
       </c>
+      <c r="M6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7">
-        <v>141</v>
+        <v>177</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H7">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7" s="1">
-        <v>45964</v>
+        <v>46062</v>
       </c>
       <c r="K7">
-        <v>-121</v>
+        <v>-91</v>
       </c>
       <c r="L7" t="s">
-        <v>25</v>
-      </c>
-      <c r="M7" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1068,28 +1119,28 @@
         <v>28</v>
       </c>
       <c r="C8">
-        <v>486</v>
+        <v>30</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="F8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>443</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J8" s="1">
-        <v>46041</v>
+        <v>46077</v>
       </c>
       <c r="K8">
-        <v>-44</v>
+        <v>-76</v>
       </c>
       <c r="L8" t="s">
         <v>29</v>
@@ -1106,302 +1157,272 @@
         <v>32</v>
       </c>
       <c r="C9">
-        <v>12</v>
+        <v>586</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>11</v>
+        <v>558</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9" s="1">
-        <v>46069</v>
+        <v>46093</v>
       </c>
       <c r="K9">
-        <v>-16</v>
+        <v>-60</v>
       </c>
       <c r="L9" t="s">
         <v>33</v>
       </c>
+      <c r="M9" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10">
-        <v>19</v>
+        <v>240</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>17</v>
+        <v>191</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J10" s="1">
-        <v>46073</v>
+        <v>46108</v>
       </c>
       <c r="K10">
-        <v>-12</v>
+        <v>-45</v>
       </c>
       <c r="L10" t="s">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="M10" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C11">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11" s="1">
-        <v>46076</v>
+        <v>46139</v>
       </c>
       <c r="K11">
-        <v>-9</v>
+        <v>-14</v>
       </c>
       <c r="L11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="M11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C12">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="H12">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
       <c r="J12" s="1">
-        <v>46104</v>
+        <v>46160</v>
       </c>
       <c r="K12">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="L12" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
         <v>0</v>
-      </c>
-      <c r="J13" s="1">
-        <v>46100</v>
-      </c>
-      <c r="K13">
-        <v>15</v>
-      </c>
-      <c r="L13" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C14">
+        <v>30</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
         <v>2</v>
       </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
-      </c>
       <c r="H14">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="I14">
         <v>0</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46097</v>
-      </c>
-      <c r="K14">
-        <v>12</v>
-      </c>
-      <c r="L14" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
         <v>50</v>
       </c>
       <c r="C15">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="I15">
         <v>0</v>
-      </c>
-      <c r="J15" s="1">
-        <v>46087</v>
-      </c>
-      <c r="K15">
-        <v>2</v>
-      </c>
-      <c r="L15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" t="s">
         <v>52</v>
       </c>
-      <c r="B16" t="s">
-        <v>53</v>
-      </c>
       <c r="C16">
-        <v>161</v>
+        <v>2</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>147</v>
+        <v>1</v>
       </c>
       <c r="I16">
         <v>0</v>
-      </c>
-      <c r="J16" s="1">
-        <v>46085</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C17">
-        <v>164</v>
+        <v>70</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F17">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>123</v>
+        <v>66</v>
       </c>
       <c r="I17">
         <v>0</v>
@@ -1409,13 +1430,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C18">
-        <v>123</v>
+        <v>37</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1424,24 +1445,27 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>17</v>
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
+        <v>57</v>
       </c>
       <c r="H18">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C19">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -1450,10 +1474,13 @@
         <v>0</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
+        <v>57</v>
       </c>
       <c r="H19">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -1461,13 +1488,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C20">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1476,10 +1503,13 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G20" t="s">
+        <v>57</v>
       </c>
       <c r="H20">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -1487,13 +1517,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C21">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -1502,10 +1532,13 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G21" t="s">
+        <v>57</v>
       </c>
       <c r="H21">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -1513,13 +1546,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -1528,10 +1561,13 @@
         <v>0</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G22" t="s">
+        <v>57</v>
       </c>
       <c r="H22">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -1539,25 +1575,28 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C23">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
+      <c r="G23" t="s">
+        <v>57</v>
+      </c>
       <c r="H23">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -1565,13 +1604,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C24">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -1583,10 +1622,10 @@
         <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H24">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -1594,13 +1633,13 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C25">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -1612,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H25">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -1623,10 +1662,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1641,7 +1680,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H26">
         <v>1</v>
@@ -1652,13 +1691,13 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1670,10 +1709,10 @@
         <v>0</v>
       </c>
       <c r="G27" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -1681,13 +1720,13 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -1699,10 +1738,10 @@
         <v>0</v>
       </c>
       <c r="G28" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -1710,10 +1749,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1728,7 +1767,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H29">
         <v>1</v>
@@ -1739,13 +1778,13 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1757,10 +1796,10 @@
         <v>0</v>
       </c>
       <c r="G30" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -1768,10 +1807,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1786,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H31">
         <v>1</v>
@@ -1797,13 +1836,13 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C32">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1815,10 +1854,10 @@
         <v>0</v>
       </c>
       <c r="G32" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H32">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -1826,13 +1865,13 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -1844,10 +1883,10 @@
         <v>0</v>
       </c>
       <c r="G33" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -1855,13 +1894,13 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -1873,10 +1912,10 @@
         <v>0</v>
       </c>
       <c r="G34" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H34">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I34">
         <v>0</v>
@@ -1884,10 +1923,10 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C35">
         <v>4</v>
@@ -1902,7 +1941,7 @@
         <v>0</v>
       </c>
       <c r="G35" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H35">
         <v>4</v>
@@ -1913,13 +1952,13 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A36" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B36" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -1931,10 +1970,10 @@
         <v>0</v>
       </c>
       <c r="G36" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H36">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I36">
         <v>0</v>
@@ -1942,13 +1981,13 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A37" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C37">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D37">
         <v>0</v>
@@ -1960,10 +1999,10 @@
         <v>0</v>
       </c>
       <c r="G37" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H37">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -1971,10 +2010,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A38" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -1989,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="G38" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -2000,13 +2039,13 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C39">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -2018,10 +2057,10 @@
         <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H39">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -2029,13 +2068,13 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A40" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -2047,10 +2086,10 @@
         <v>0</v>
       </c>
       <c r="G40" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I40">
         <v>0</v>
@@ -2058,13 +2097,13 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A41" t="s">
-        <v>31</v>
+        <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -2076,10 +2115,10 @@
         <v>0</v>
       </c>
       <c r="G41" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H41">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="I41">
         <v>0</v>
@@ -2087,10 +2126,10 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A42" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -2105,7 +2144,7 @@
         <v>0</v>
       </c>
       <c r="G42" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H42">
         <v>1</v>
@@ -2116,13 +2155,13 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A43" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -2134,10 +2173,10 @@
         <v>0</v>
       </c>
       <c r="G43" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -2145,13 +2184,13 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C44">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -2163,10 +2202,10 @@
         <v>0</v>
       </c>
       <c r="G44" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H44">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -2174,10 +2213,10 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2192,7 +2231,7 @@
         <v>0</v>
       </c>
       <c r="G45" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H45">
         <v>1</v>
@@ -2203,10 +2242,10 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -2221,7 +2260,7 @@
         <v>0</v>
       </c>
       <c r="G46" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -2232,13 +2271,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C47">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -2250,10 +2289,10 @@
         <v>0</v>
       </c>
       <c r="G47" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H47">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="I47">
         <v>0</v>
@@ -2261,13 +2300,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C48">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -2279,10 +2318,10 @@
         <v>0</v>
       </c>
       <c r="G48" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H48">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="I48">
         <v>0</v>
@@ -2290,13 +2329,13 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B49" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -2308,10 +2347,10 @@
         <v>0</v>
       </c>
       <c r="G49" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H49">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="I49">
         <v>0</v>
@@ -2319,13 +2358,13 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B50" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -2337,10 +2376,10 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50">
         <v>0</v>
@@ -2348,13 +2387,13 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A51" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B51" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -2366,10 +2405,10 @@
         <v>0</v>
       </c>
       <c r="G51" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
         <v>0</v>
@@ -2377,10 +2416,10 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A52" t="s">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C52">
         <v>10</v>
@@ -2395,7 +2434,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H52">
         <v>10</v>
@@ -2406,13 +2445,13 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A53" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B53" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C53">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D53">
         <v>0</v>
@@ -2424,10 +2463,10 @@
         <v>0</v>
       </c>
       <c r="G53" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I53">
         <v>0</v>
@@ -2435,13 +2474,13 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A54" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C54">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -2453,10 +2492,10 @@
         <v>0</v>
       </c>
       <c r="G54" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H54">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="I54">
         <v>0</v>
@@ -2464,13 +2503,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A55" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B55" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C55">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -2482,10 +2521,10 @@
         <v>0</v>
       </c>
       <c r="G55" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H55">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I55">
         <v>0</v>
@@ -2493,13 +2532,13 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A56" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B56" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -2511,10 +2550,10 @@
         <v>0</v>
       </c>
       <c r="G56" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I56">
         <v>0</v>
@@ -2522,13 +2561,13 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>43</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C57">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -2540,10 +2579,10 @@
         <v>0</v>
       </c>
       <c r="G57" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H57">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="I57">
         <v>0</v>
@@ -2551,10 +2590,10 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A58" t="s">
-        <v>111</v>
+        <v>43</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2569,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="G58" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H58">
         <v>1</v>
@@ -2580,13 +2619,13 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A59" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B59" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -2598,10 +2637,10 @@
         <v>0</v>
       </c>
       <c r="G59" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I59">
         <v>0</v>
@@ -2609,10 +2648,10 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="B60" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -2627,7 +2666,7 @@
         <v>0</v>
       </c>
       <c r="G60" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H60">
         <v>1</v>
@@ -2638,13 +2677,13 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="B61" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -2656,10 +2695,10 @@
         <v>0</v>
       </c>
       <c r="G61" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I61">
         <v>0</v>
@@ -2667,13 +2706,13 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A62" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B62" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C62">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -2685,10 +2724,10 @@
         <v>0</v>
       </c>
       <c r="G62" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H62">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I62">
         <v>0</v>
@@ -2696,13 +2735,13 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A63" t="s">
-        <v>118</v>
+        <v>46</v>
       </c>
       <c r="B63" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C63">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -2714,10 +2753,10 @@
         <v>0</v>
       </c>
       <c r="G63" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H63">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="I63">
         <v>0</v>
@@ -2725,13 +2764,13 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A64" t="s">
-        <v>118</v>
+        <v>46</v>
       </c>
       <c r="B64" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -2743,10 +2782,10 @@
         <v>0</v>
       </c>
       <c r="G64" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I64">
         <v>0</v>
@@ -2754,13 +2793,13 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A65" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B65" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C65">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="D65">
         <v>0</v>
@@ -2772,10 +2811,10 @@
         <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H65">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="I65">
         <v>0</v>
@@ -2783,10 +2822,10 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A66" t="s">
-        <v>43</v>
+        <v>116</v>
       </c>
       <c r="B66" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C66">
         <v>1</v>
@@ -2801,7 +2840,7 @@
         <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H66">
         <v>1</v>
@@ -2812,13 +2851,13 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A67" t="s">
-        <v>43</v>
+        <v>118</v>
       </c>
       <c r="B67" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C67">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D67">
         <v>0</v>
@@ -2830,10 +2869,10 @@
         <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H67">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I67">
         <v>0</v>
@@ -2841,13 +2880,13 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A68" t="s">
-        <v>43</v>
+        <v>120</v>
       </c>
       <c r="B68" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C68">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D68">
         <v>0</v>
@@ -2859,10 +2898,10 @@
         <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H68">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I68">
         <v>0</v>
@@ -2870,13 +2909,13 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A69" t="s">
-        <v>43</v>
+        <v>120</v>
       </c>
       <c r="B69" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D69">
         <v>0</v>
@@ -2888,10 +2927,10 @@
         <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I69">
         <v>0</v>
@@ -2899,13 +2938,13 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A70" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="B70" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C70">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="D70">
         <v>0</v>
@@ -2917,10 +2956,10 @@
         <v>0</v>
       </c>
       <c r="G70" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H70">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="I70">
         <v>0</v>
@@ -2928,10 +2967,10 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A71" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="B71" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -2946,7 +2985,7 @@
         <v>0</v>
       </c>
       <c r="G71" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H71">
         <v>1</v>
@@ -2957,13 +2996,13 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A72" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B72" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D72">
         <v>0</v>
@@ -2975,10 +3014,10 @@
         <v>0</v>
       </c>
       <c r="G72" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I72">
         <v>0</v>
@@ -2986,13 +3025,13 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A73" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B73" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D73">
         <v>0</v>
@@ -3004,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="G73" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I73">
         <v>0</v>
@@ -3015,10 +3054,10 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A74" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="B74" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -3033,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="G74" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H74">
         <v>1</v>
@@ -3044,10 +3083,10 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A75" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B75" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -3062,7 +3101,7 @@
         <v>0</v>
       </c>
       <c r="G75" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H75">
         <v>1</v>
@@ -3073,13 +3112,13 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A76" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="B76" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C76">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D76">
         <v>0</v>
@@ -3091,10 +3130,10 @@
         <v>0</v>
       </c>
       <c r="G76" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H76">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I76">
         <v>0</v>
@@ -3102,13 +3141,13 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A77" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="B77" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D77">
         <v>0</v>
@@ -3120,10 +3159,10 @@
         <v>0</v>
       </c>
       <c r="G77" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I77">
         <v>0</v>
@@ -3131,13 +3170,13 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A78" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="B78" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78">
         <v>0</v>
@@ -3149,10 +3188,10 @@
         <v>0</v>
       </c>
       <c r="G78" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78">
         <v>0</v>
@@ -3160,10 +3199,10 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A79" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B79" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C79">
         <v>2</v>
@@ -3178,7 +3217,7 @@
         <v>0</v>
       </c>
       <c r="G79" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H79">
         <v>2</v>
@@ -3189,13 +3228,13 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A80" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B80" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C80">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D80">
         <v>0</v>
@@ -3207,10 +3246,10 @@
         <v>0</v>
       </c>
       <c r="G80" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H80">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I80">
         <v>0</v>
@@ -3218,13 +3257,13 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A81" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="B81" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C81">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="D81">
         <v>0</v>
@@ -3236,10 +3275,10 @@
         <v>0</v>
       </c>
       <c r="G81" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H81">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="I81">
         <v>0</v>
@@ -3247,13 +3286,13 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A82" t="s">
-        <v>65</v>
+        <v>138</v>
       </c>
       <c r="B82" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C82">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="D82">
         <v>0</v>
@@ -3265,10 +3304,10 @@
         <v>0</v>
       </c>
       <c r="G82" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H82">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="I82">
         <v>0</v>
@@ -3276,10 +3315,10 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A83" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B83" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -3294,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="G83" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H83">
         <v>1</v>
@@ -3305,13 +3344,13 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A84" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B84" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="C84">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D84">
         <v>0</v>
@@ -3323,10 +3362,10 @@
         <v>0</v>
       </c>
       <c r="G84" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H84">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="I84">
         <v>0</v>
@@ -3334,10 +3373,10 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A85" t="s">
-        <v>49</v>
+        <v>144</v>
       </c>
       <c r="B85" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C85">
         <v>1</v>
@@ -3352,7 +3391,7 @@
         <v>0</v>
       </c>
       <c r="G85" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H85">
         <v>1</v>
@@ -3363,30 +3402,407 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A86" t="s">
-        <v>49</v>
+        <v>146</v>
       </c>
       <c r="B86" t="s">
+        <v>147</v>
+      </c>
+      <c r="C86">
+        <v>2</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="G86" t="s">
+        <v>57</v>
+      </c>
+      <c r="H86">
+        <v>2</v>
+      </c>
+      <c r="I86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A87" t="s">
+        <v>146</v>
+      </c>
+      <c r="B87" t="s">
+        <v>148</v>
+      </c>
+      <c r="C87">
+        <v>2</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87" t="s">
+        <v>57</v>
+      </c>
+      <c r="H87">
+        <v>2</v>
+      </c>
+      <c r="I87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A88" t="s">
+        <v>149</v>
+      </c>
+      <c r="B88" t="s">
+        <v>150</v>
+      </c>
+      <c r="C88">
+        <v>9</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88" t="s">
+        <v>57</v>
+      </c>
+      <c r="H88">
+        <v>9</v>
+      </c>
+      <c r="I88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A89" t="s">
+        <v>151</v>
+      </c>
+      <c r="B89" t="s">
         <v>152</v>
       </c>
-      <c r="C86">
-        <v>1</v>
-      </c>
-      <c r="D86">
-        <v>0</v>
-      </c>
-      <c r="E86">
-        <v>0</v>
-      </c>
-      <c r="F86">
-        <v>0</v>
-      </c>
-      <c r="G86" t="s">
-        <v>70</v>
-      </c>
-      <c r="H86">
-        <v>1</v>
-      </c>
-      <c r="I86">
+      <c r="C89">
+        <v>136</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+      <c r="F89">
+        <v>0</v>
+      </c>
+      <c r="G89" t="s">
+        <v>57</v>
+      </c>
+      <c r="H89">
+        <v>136</v>
+      </c>
+      <c r="I89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A90" t="s">
+        <v>153</v>
+      </c>
+      <c r="B90" t="s">
+        <v>154</v>
+      </c>
+      <c r="C90">
+        <v>2</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+      <c r="G90" t="s">
+        <v>57</v>
+      </c>
+      <c r="H90">
+        <v>2</v>
+      </c>
+      <c r="I90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A91" t="s">
+        <v>155</v>
+      </c>
+      <c r="B91" t="s">
+        <v>156</v>
+      </c>
+      <c r="C91">
+        <v>9</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="G91" t="s">
+        <v>57</v>
+      </c>
+      <c r="H91">
+        <v>9</v>
+      </c>
+      <c r="I91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A92" t="s">
+        <v>157</v>
+      </c>
+      <c r="B92" t="s">
+        <v>158</v>
+      </c>
+      <c r="C92">
+        <v>16</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>0</v>
+      </c>
+      <c r="G92" t="s">
+        <v>57</v>
+      </c>
+      <c r="H92">
+        <v>16</v>
+      </c>
+      <c r="I92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A93" t="s">
+        <v>157</v>
+      </c>
+      <c r="B93" t="s">
+        <v>159</v>
+      </c>
+      <c r="C93">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93">
+        <v>0</v>
+      </c>
+      <c r="G93" t="s">
+        <v>57</v>
+      </c>
+      <c r="H93">
+        <v>24</v>
+      </c>
+      <c r="I93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A94" t="s">
+        <v>160</v>
+      </c>
+      <c r="B94" t="s">
+        <v>161</v>
+      </c>
+      <c r="C94">
+        <v>170</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
+        <v>0</v>
+      </c>
+      <c r="F94">
+        <v>0</v>
+      </c>
+      <c r="G94" t="s">
+        <v>57</v>
+      </c>
+      <c r="H94">
+        <v>170</v>
+      </c>
+      <c r="I94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A95" t="s">
+        <v>162</v>
+      </c>
+      <c r="B95" t="s">
+        <v>163</v>
+      </c>
+      <c r="C95">
+        <v>1</v>
+      </c>
+      <c r="D95">
+        <v>0</v>
+      </c>
+      <c r="E95">
+        <v>0</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+      <c r="G95" t="s">
+        <v>57</v>
+      </c>
+      <c r="H95">
+        <v>1</v>
+      </c>
+      <c r="I95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A96" t="s">
+        <v>164</v>
+      </c>
+      <c r="B96" t="s">
+        <v>165</v>
+      </c>
+      <c r="C96">
+        <v>15</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="G96" t="s">
+        <v>57</v>
+      </c>
+      <c r="H96">
+        <v>15</v>
+      </c>
+      <c r="I96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A97" t="s">
+        <v>166</v>
+      </c>
+      <c r="B97" t="s">
+        <v>167</v>
+      </c>
+      <c r="C97">
+        <v>1</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="G97" t="s">
+        <v>57</v>
+      </c>
+      <c r="H97">
+        <v>1</v>
+      </c>
+      <c r="I97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A98" t="s">
+        <v>166</v>
+      </c>
+      <c r="B98" t="s">
+        <v>168</v>
+      </c>
+      <c r="C98">
+        <v>1</v>
+      </c>
+      <c r="D98">
+        <v>0</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="G98" t="s">
+        <v>57</v>
+      </c>
+      <c r="H98">
+        <v>1</v>
+      </c>
+      <c r="I98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A99" t="s">
+        <v>166</v>
+      </c>
+      <c r="B99" t="s">
+        <v>169</v>
+      </c>
+      <c r="C99">
+        <v>12</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+      <c r="G99" t="s">
+        <v>57</v>
+      </c>
+      <c r="H99">
+        <v>12</v>
+      </c>
+      <c r="I99">
         <v>0</v>
       </c>
     </row>

</xml_diff>